<commit_message>
&&& - 86984492 от 15.03.2026 https://meshok.net/ - 86922915 от 13.03.2026 https://meshok.net/
</commit_message>
<xml_diff>
--- a/Collections/Canada/#Canada#Regular#[1953-present]#circulation_quality.xlsx
+++ b/Collections/Canada/#Canada#Regular#[1953-present]#circulation_quality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\Canada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C97E8D3-5EE5-45EA-AC35-FBB146FD40BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B6495B-1D47-4867-AF11-0A2EEC16B9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1¢" sheetId="3" r:id="rId1"/>
@@ -9101,7 +9101,7 @@
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I65 I62 I70:I73 I67">
+  <conditionalFormatting sqref="I62 I65 I70:I73 I67">
     <cfRule type="colorScale" priority="102">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -14114,7 +14114,7 @@
         <v>0</v>
       </c>
       <c r="J30" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>0</v>

</xml_diff>